<commit_message>
test and harden workbench
</commit_message>
<xml_diff>
--- a/outputs/01a014e4-2b3b-7f43-9fa3-d1086c95abc9/船期自动抓取模板.xlsx
+++ b/outputs/01a014e4-2b3b-7f43-9fa3-d1086c95abc9/船期自动抓取模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="船期追踪" sheetId="1" r:id="R3a391c4f19f5456c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="船司规则" sheetId="2" r:id="Rf0ef7d36cbd44a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="船期追踪" sheetId="1" r:id="R92e370501b1d4cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="船司规则" sheetId="2" r:id="Rc0fae9e95c914d8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -322,17 +322,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ShipmentTrackingTable" displayName="ShipmentTrackingTable" ref="A1:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ShipmentTrackingTable" displayName="ShipmentTrackingTable" ref="A1:J16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="船司"/>
     <x:tableColumn id="2" name="到港时间"/>
     <x:tableColumn id="3" name="提单号"/>
     <x:tableColumn id="4" name="柜号"/>
     <x:tableColumn id="5" name="卸船时间"/>
     <x:tableColumn id="6" name="船只状态"/>
-    <x:tableColumn id="7" name="最后更新时间"/>
-    <x:tableColumn id="8" name="备注"/>
-    <x:tableColumn id="9" name="进度"/>
+    <x:tableColumn id="7" name="人工标记"/>
+    <x:tableColumn id="8" name="最后更新时间"/>
+    <x:tableColumn id="9" name="备注"/>
+    <x:tableColumn id="10" name="进度"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -553,9 +554,10 @@
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="36" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="36" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -578,12 +580,15 @@
         <x:v>船只状态</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
+        <x:v>人工标记</x:v>
+      </x:c>
+      <x:c r="H1" s="10" t="str">
         <x:v>最后更新时间</x:v>
       </x:c>
-      <x:c r="H1" s="10" t="str">
+      <x:c r="I1" s="10" t="str">
         <x:v>备注</x:v>
       </x:c>
-      <x:c r="I1" s="11" t="str">
+      <x:c r="J1" s="11" t="str">
         <x:v>进度</x:v>
       </x:c>
     </x:row>
@@ -604,11 +609,12 @@
       <x:c r="F2" s="19" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G2" s="22" t="str"/>
-      <x:c r="H2" s="32" t="str">
+      <x:c r="G2" s="19" t="str"/>
+      <x:c r="H2" s="22" t="str"/>
+      <x:c r="I2" s="32" t="str">
         <x:v>真实订单，运行时请求 OOCL 官方接口</x:v>
       </x:c>
-      <x:c r="I2" s="19" t="str">
+      <x:c r="J2" s="19" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -629,11 +635,12 @@
       <x:c r="F3" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str"/>
-      <x:c r="H3" s="33" t="str">
+      <x:c r="G3" s="17" t="str"/>
+      <x:c r="H3" s="23" t="str"/>
+      <x:c r="I3" s="33" t="str">
         <x:v>真实订单，已接入官方三段追踪查询</x:v>
       </x:c>
-      <x:c r="I3" s="17" t="str">
+      <x:c r="J3" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -654,11 +661,12 @@
       <x:c r="F4" s="20" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G4" s="24" t="str"/>
-      <x:c r="H4" s="34" t="str">
+      <x:c r="G4" s="20" t="str"/>
+      <x:c r="H4" s="24" t="str"/>
+      <x:c r="I4" s="34" t="str">
         <x:v>提单号和柜号分别查询后合并</x:v>
       </x:c>
-      <x:c r="I4" s="20" t="str">
+      <x:c r="J4" s="20" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -679,11 +687,12 @@
       <x:c r="F5" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G5" s="23" t="str"/>
-      <x:c r="H5" s="33" t="str">
+      <x:c r="G5" s="17" t="str"/>
+      <x:c r="H5" s="23" t="str"/>
+      <x:c r="I5" s="33" t="str">
         <x:v>真实订单，运行时请求官网并记录风控原因</x:v>
       </x:c>
-      <x:c r="I5" s="17" t="str">
+      <x:c r="J5" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -704,11 +713,12 @@
       <x:c r="F6" s="20" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G6" s="24" t="str"/>
-      <x:c r="H6" s="34" t="str">
+      <x:c r="G6" s="20" t="str"/>
+      <x:c r="H6" s="24" t="str"/>
+      <x:c r="I6" s="34" t="str">
         <x:v>真实订单，已接入官网解析器</x:v>
       </x:c>
-      <x:c r="I6" s="20" t="str">
+      <x:c r="J6" s="20" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -729,11 +739,12 @@
       <x:c r="F7" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G7" s="23" t="str"/>
-      <x:c r="H7" s="33" t="str">
+      <x:c r="G7" s="17" t="str"/>
+      <x:c r="H7" s="23" t="str"/>
+      <x:c r="I7" s="33" t="str">
         <x:v>真实订单，运行时请求官网并记录真实响应</x:v>
       </x:c>
-      <x:c r="I7" s="17" t="str">
+      <x:c r="J7" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -754,11 +765,12 @@
       <x:c r="F8" s="20" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G8" s="24" t="str"/>
-      <x:c r="H8" s="34" t="str">
+      <x:c r="G8" s="20" t="str"/>
+      <x:c r="H8" s="24" t="str"/>
+      <x:c r="I8" s="34" t="str">
         <x:v>真实订单，已接入官方公开接口</x:v>
       </x:c>
-      <x:c r="I8" s="20" t="str">
+      <x:c r="J8" s="20" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -779,11 +791,12 @@
       <x:c r="F9" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G9" s="23" t="str"/>
-      <x:c r="H9" s="33" t="str">
+      <x:c r="G9" s="17" t="str"/>
+      <x:c r="H9" s="23" t="str"/>
+      <x:c r="I9" s="33" t="str">
         <x:v>真实订单，运行时请求官网并记录风控原因</x:v>
       </x:c>
-      <x:c r="I9" s="17" t="str">
+      <x:c r="J9" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -804,11 +817,12 @@
       <x:c r="F10" s="20" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G10" s="24" t="str"/>
-      <x:c r="H10" s="34" t="str">
+      <x:c r="G10" s="20" t="str"/>
+      <x:c r="H10" s="24" t="str"/>
+      <x:c r="I10" s="34" t="str">
         <x:v>MAEU 固定对应马士基</x:v>
       </x:c>
-      <x:c r="I10" s="20" t="str">
+      <x:c r="J10" s="20" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -829,11 +843,12 @@
       <x:c r="F11" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G11" s="23" t="str"/>
-      <x:c r="H11" s="33" t="str">
+      <x:c r="G11" s="17" t="str"/>
+      <x:c r="H11" s="23" t="str"/>
+      <x:c r="I11" s="33" t="str">
         <x:v>真实订单，已接入提单与货柜动态查询</x:v>
       </x:c>
-      <x:c r="I11" s="17" t="str">
+      <x:c r="J11" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -854,11 +869,12 @@
       <x:c r="F12" s="20" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G12" s="24" t="str"/>
-      <x:c r="H12" s="34" t="str">
+      <x:c r="G12" s="20" t="str"/>
+      <x:c r="H12" s="24" t="str"/>
+      <x:c r="I12" s="34" t="str">
         <x:v>真实订单，运行时请求官网并记录真实响应</x:v>
       </x:c>
-      <x:c r="I12" s="20" t="str">
+      <x:c r="J12" s="20" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -879,11 +895,12 @@
       <x:c r="F13" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G13" s="23" t="str"/>
-      <x:c r="H13" s="33" t="str">
+      <x:c r="G13" s="17" t="str"/>
+      <x:c r="H13" s="23" t="str"/>
+      <x:c r="I13" s="33" t="str">
         <x:v>真实订单，运行时请求官网并记录风控原因</x:v>
       </x:c>
-      <x:c r="I13" s="17" t="str">
+      <x:c r="J13" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -904,11 +921,12 @@
       <x:c r="F14" s="20" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G14" s="24" t="str"/>
-      <x:c r="H14" s="34" t="str">
+      <x:c r="G14" s="20" t="str"/>
+      <x:c r="H14" s="24" t="str"/>
+      <x:c r="I14" s="34" t="str">
         <x:v>MEDU 固定对应地中海</x:v>
       </x:c>
-      <x:c r="I14" s="20" t="str">
+      <x:c r="J14" s="20" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -929,11 +947,12 @@
       <x:c r="F15" s="17" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G15" s="23" t="str"/>
-      <x:c r="H15" s="33" t="str">
+      <x:c r="G15" s="17" t="str"/>
+      <x:c r="H15" s="23" t="str"/>
+      <x:c r="I15" s="33" t="str">
         <x:v>真实订单，运行时请求官网并记录真实响应</x:v>
       </x:c>
-      <x:c r="I15" s="17" t="str">
+      <x:c r="J15" s="17" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -954,11 +973,12 @@
       <x:c r="F16" s="21" t="str">
         <x:v>未到港未卸船</x:v>
       </x:c>
-      <x:c r="G16" s="25" t="str"/>
-      <x:c r="H16" s="35" t="str">
+      <x:c r="G16" s="21" t="str"/>
+      <x:c r="H16" s="25" t="str"/>
+      <x:c r="I16" s="35" t="str">
         <x:v>真实订单，运行时请求官网并记录真实响应</x:v>
       </x:c>
-      <x:c r="I16" s="21" t="str">
+      <x:c r="J16" s="21" t="str">
         <x:v>待查询</x:v>
       </x:c>
     </x:row>
@@ -967,1479 +987,1479 @@
       <x:c r="C17" s="31"/>
       <x:c r="D17" s="31"/>
       <x:c r="E17" s="26"/>
-      <x:c r="G17" s="26"/>
-      <x:c r="H17" s="36"/>
+      <x:c r="H17" s="26"/>
+      <x:c r="I17" s="36"/>
     </x:row>
     <x:row r="18">
       <x:c r="B18" s="26"/>
       <x:c r="C18" s="31"/>
       <x:c r="D18" s="31"/>
       <x:c r="E18" s="26"/>
-      <x:c r="G18" s="26"/>
-      <x:c r="H18" s="36"/>
+      <x:c r="H18" s="26"/>
+      <x:c r="I18" s="36"/>
     </x:row>
     <x:row r="19">
       <x:c r="B19" s="26"/>
       <x:c r="C19" s="31"/>
       <x:c r="D19" s="31"/>
       <x:c r="E19" s="26"/>
-      <x:c r="G19" s="26"/>
-      <x:c r="H19" s="36"/>
+      <x:c r="H19" s="26"/>
+      <x:c r="I19" s="36"/>
     </x:row>
     <x:row r="20">
       <x:c r="B20" s="26"/>
       <x:c r="C20" s="31"/>
       <x:c r="D20" s="31"/>
       <x:c r="E20" s="26"/>
-      <x:c r="G20" s="26"/>
-      <x:c r="H20" s="36"/>
+      <x:c r="H20" s="26"/>
+      <x:c r="I20" s="36"/>
     </x:row>
     <x:row r="21">
       <x:c r="B21" s="26"/>
       <x:c r="C21" s="31"/>
       <x:c r="D21" s="31"/>
       <x:c r="E21" s="26"/>
-      <x:c r="G21" s="26"/>
-      <x:c r="H21" s="36"/>
+      <x:c r="H21" s="26"/>
+      <x:c r="I21" s="36"/>
     </x:row>
     <x:row r="22">
       <x:c r="B22" s="26"/>
       <x:c r="C22" s="31"/>
       <x:c r="D22" s="31"/>
       <x:c r="E22" s="26"/>
-      <x:c r="G22" s="26"/>
-      <x:c r="H22" s="36"/>
+      <x:c r="H22" s="26"/>
+      <x:c r="I22" s="36"/>
     </x:row>
     <x:row r="23">
       <x:c r="B23" s="26"/>
       <x:c r="C23" s="31"/>
       <x:c r="D23" s="31"/>
       <x:c r="E23" s="26"/>
-      <x:c r="G23" s="26"/>
-      <x:c r="H23" s="36"/>
+      <x:c r="H23" s="26"/>
+      <x:c r="I23" s="36"/>
     </x:row>
     <x:row r="24">
       <x:c r="B24" s="26"/>
       <x:c r="C24" s="31"/>
       <x:c r="D24" s="31"/>
       <x:c r="E24" s="26"/>
-      <x:c r="G24" s="26"/>
-      <x:c r="H24" s="36"/>
+      <x:c r="H24" s="26"/>
+      <x:c r="I24" s="36"/>
     </x:row>
     <x:row r="25">
       <x:c r="B25" s="26"/>
       <x:c r="C25" s="31"/>
       <x:c r="D25" s="31"/>
       <x:c r="E25" s="26"/>
-      <x:c r="G25" s="26"/>
-      <x:c r="H25" s="36"/>
+      <x:c r="H25" s="26"/>
+      <x:c r="I25" s="36"/>
     </x:row>
     <x:row r="26">
       <x:c r="B26" s="26"/>
       <x:c r="C26" s="31"/>
       <x:c r="D26" s="31"/>
       <x:c r="E26" s="26"/>
-      <x:c r="G26" s="26"/>
-      <x:c r="H26" s="36"/>
+      <x:c r="H26" s="26"/>
+      <x:c r="I26" s="36"/>
     </x:row>
     <x:row r="27">
       <x:c r="B27" s="26"/>
       <x:c r="C27" s="31"/>
       <x:c r="D27" s="31"/>
       <x:c r="E27" s="26"/>
-      <x:c r="G27" s="26"/>
-      <x:c r="H27" s="36"/>
+      <x:c r="H27" s="26"/>
+      <x:c r="I27" s="36"/>
     </x:row>
     <x:row r="28">
       <x:c r="B28" s="26"/>
       <x:c r="C28" s="31"/>
       <x:c r="D28" s="31"/>
       <x:c r="E28" s="26"/>
-      <x:c r="G28" s="26"/>
-      <x:c r="H28" s="36"/>
+      <x:c r="H28" s="26"/>
+      <x:c r="I28" s="36"/>
     </x:row>
     <x:row r="29">
       <x:c r="B29" s="26"/>
       <x:c r="C29" s="31"/>
       <x:c r="D29" s="31"/>
       <x:c r="E29" s="26"/>
-      <x:c r="G29" s="26"/>
-      <x:c r="H29" s="36"/>
+      <x:c r="H29" s="26"/>
+      <x:c r="I29" s="36"/>
     </x:row>
     <x:row r="30">
       <x:c r="B30" s="26"/>
       <x:c r="C30" s="31"/>
       <x:c r="D30" s="31"/>
       <x:c r="E30" s="26"/>
-      <x:c r="G30" s="26"/>
-      <x:c r="H30" s="36"/>
+      <x:c r="H30" s="26"/>
+      <x:c r="I30" s="36"/>
     </x:row>
     <x:row r="31">
       <x:c r="B31" s="26"/>
       <x:c r="C31" s="31"/>
       <x:c r="D31" s="31"/>
       <x:c r="E31" s="26"/>
-      <x:c r="G31" s="26"/>
-      <x:c r="H31" s="36"/>
+      <x:c r="H31" s="26"/>
+      <x:c r="I31" s="36"/>
     </x:row>
     <x:row r="32">
       <x:c r="B32" s="26"/>
       <x:c r="C32" s="31"/>
       <x:c r="D32" s="31"/>
       <x:c r="E32" s="26"/>
-      <x:c r="G32" s="26"/>
-      <x:c r="H32" s="36"/>
+      <x:c r="H32" s="26"/>
+      <x:c r="I32" s="36"/>
     </x:row>
     <x:row r="33">
       <x:c r="B33" s="26"/>
       <x:c r="C33" s="31"/>
       <x:c r="D33" s="31"/>
       <x:c r="E33" s="26"/>
-      <x:c r="G33" s="26"/>
-      <x:c r="H33" s="36"/>
+      <x:c r="H33" s="26"/>
+      <x:c r="I33" s="36"/>
     </x:row>
     <x:row r="34">
       <x:c r="B34" s="26"/>
       <x:c r="C34" s="31"/>
       <x:c r="D34" s="31"/>
       <x:c r="E34" s="26"/>
-      <x:c r="G34" s="26"/>
-      <x:c r="H34" s="36"/>
+      <x:c r="H34" s="26"/>
+      <x:c r="I34" s="36"/>
     </x:row>
     <x:row r="35">
       <x:c r="B35" s="26"/>
       <x:c r="C35" s="31"/>
       <x:c r="D35" s="31"/>
       <x:c r="E35" s="26"/>
-      <x:c r="G35" s="26"/>
-      <x:c r="H35" s="36"/>
+      <x:c r="H35" s="26"/>
+      <x:c r="I35" s="36"/>
     </x:row>
     <x:row r="36">
       <x:c r="B36" s="26"/>
       <x:c r="C36" s="31"/>
       <x:c r="D36" s="31"/>
       <x:c r="E36" s="26"/>
-      <x:c r="G36" s="26"/>
-      <x:c r="H36" s="36"/>
+      <x:c r="H36" s="26"/>
+      <x:c r="I36" s="36"/>
     </x:row>
     <x:row r="37">
       <x:c r="B37" s="26"/>
       <x:c r="C37" s="31"/>
       <x:c r="D37" s="31"/>
       <x:c r="E37" s="26"/>
-      <x:c r="G37" s="26"/>
-      <x:c r="H37" s="36"/>
+      <x:c r="H37" s="26"/>
+      <x:c r="I37" s="36"/>
     </x:row>
     <x:row r="38">
       <x:c r="B38" s="26"/>
       <x:c r="C38" s="31"/>
       <x:c r="D38" s="31"/>
       <x:c r="E38" s="26"/>
-      <x:c r="G38" s="26"/>
-      <x:c r="H38" s="36"/>
+      <x:c r="H38" s="26"/>
+      <x:c r="I38" s="36"/>
     </x:row>
     <x:row r="39">
       <x:c r="B39" s="26"/>
       <x:c r="C39" s="31"/>
       <x:c r="D39" s="31"/>
       <x:c r="E39" s="26"/>
-      <x:c r="G39" s="26"/>
-      <x:c r="H39" s="36"/>
+      <x:c r="H39" s="26"/>
+      <x:c r="I39" s="36"/>
     </x:row>
     <x:row r="40">
       <x:c r="B40" s="26"/>
       <x:c r="C40" s="31"/>
       <x:c r="D40" s="31"/>
       <x:c r="E40" s="26"/>
-      <x:c r="G40" s="26"/>
-      <x:c r="H40" s="36"/>
+      <x:c r="H40" s="26"/>
+      <x:c r="I40" s="36"/>
     </x:row>
     <x:row r="41">
       <x:c r="B41" s="26"/>
       <x:c r="C41" s="31"/>
       <x:c r="D41" s="31"/>
       <x:c r="E41" s="26"/>
-      <x:c r="G41" s="26"/>
-      <x:c r="H41" s="36"/>
+      <x:c r="H41" s="26"/>
+      <x:c r="I41" s="36"/>
     </x:row>
     <x:row r="42">
       <x:c r="B42" s="26"/>
       <x:c r="C42" s="31"/>
       <x:c r="D42" s="31"/>
       <x:c r="E42" s="26"/>
-      <x:c r="G42" s="26"/>
-      <x:c r="H42" s="36"/>
+      <x:c r="H42" s="26"/>
+      <x:c r="I42" s="36"/>
     </x:row>
     <x:row r="43">
       <x:c r="B43" s="26"/>
       <x:c r="C43" s="31"/>
       <x:c r="D43" s="31"/>
       <x:c r="E43" s="26"/>
-      <x:c r="G43" s="26"/>
-      <x:c r="H43" s="36"/>
+      <x:c r="H43" s="26"/>
+      <x:c r="I43" s="36"/>
     </x:row>
     <x:row r="44">
       <x:c r="B44" s="26"/>
       <x:c r="C44" s="31"/>
       <x:c r="D44" s="31"/>
       <x:c r="E44" s="26"/>
-      <x:c r="G44" s="26"/>
-      <x:c r="H44" s="36"/>
+      <x:c r="H44" s="26"/>
+      <x:c r="I44" s="36"/>
     </x:row>
     <x:row r="45">
       <x:c r="B45" s="26"/>
       <x:c r="C45" s="31"/>
       <x:c r="D45" s="31"/>
       <x:c r="E45" s="26"/>
-      <x:c r="G45" s="26"/>
-      <x:c r="H45" s="36"/>
+      <x:c r="H45" s="26"/>
+      <x:c r="I45" s="36"/>
     </x:row>
     <x:row r="46">
       <x:c r="B46" s="26"/>
       <x:c r="C46" s="31"/>
       <x:c r="D46" s="31"/>
       <x:c r="E46" s="26"/>
-      <x:c r="G46" s="26"/>
-      <x:c r="H46" s="36"/>
+      <x:c r="H46" s="26"/>
+      <x:c r="I46" s="36"/>
     </x:row>
     <x:row r="47">
       <x:c r="B47" s="26"/>
       <x:c r="C47" s="31"/>
       <x:c r="D47" s="31"/>
       <x:c r="E47" s="26"/>
-      <x:c r="G47" s="26"/>
-      <x:c r="H47" s="36"/>
+      <x:c r="H47" s="26"/>
+      <x:c r="I47" s="36"/>
     </x:row>
     <x:row r="48">
       <x:c r="B48" s="26"/>
       <x:c r="C48" s="31"/>
       <x:c r="D48" s="31"/>
       <x:c r="E48" s="26"/>
-      <x:c r="G48" s="26"/>
-      <x:c r="H48" s="36"/>
+      <x:c r="H48" s="26"/>
+      <x:c r="I48" s="36"/>
     </x:row>
     <x:row r="49">
       <x:c r="B49" s="26"/>
       <x:c r="C49" s="31"/>
       <x:c r="D49" s="31"/>
       <x:c r="E49" s="26"/>
-      <x:c r="G49" s="26"/>
-      <x:c r="H49" s="36"/>
+      <x:c r="H49" s="26"/>
+      <x:c r="I49" s="36"/>
     </x:row>
     <x:row r="50">
       <x:c r="B50" s="26"/>
       <x:c r="C50" s="31"/>
       <x:c r="D50" s="31"/>
       <x:c r="E50" s="26"/>
-      <x:c r="G50" s="26"/>
-      <x:c r="H50" s="36"/>
+      <x:c r="H50" s="26"/>
+      <x:c r="I50" s="36"/>
     </x:row>
     <x:row r="51">
       <x:c r="B51" s="26"/>
       <x:c r="C51" s="31"/>
       <x:c r="D51" s="31"/>
       <x:c r="E51" s="26"/>
-      <x:c r="G51" s="26"/>
-      <x:c r="H51" s="36"/>
+      <x:c r="H51" s="26"/>
+      <x:c r="I51" s="36"/>
     </x:row>
     <x:row r="52">
       <x:c r="B52" s="26"/>
       <x:c r="C52" s="31"/>
       <x:c r="D52" s="31"/>
       <x:c r="E52" s="26"/>
-      <x:c r="G52" s="26"/>
-      <x:c r="H52" s="36"/>
+      <x:c r="H52" s="26"/>
+      <x:c r="I52" s="36"/>
     </x:row>
     <x:row r="53">
       <x:c r="B53" s="26"/>
       <x:c r="C53" s="31"/>
       <x:c r="D53" s="31"/>
       <x:c r="E53" s="26"/>
-      <x:c r="G53" s="26"/>
-      <x:c r="H53" s="36"/>
+      <x:c r="H53" s="26"/>
+      <x:c r="I53" s="36"/>
     </x:row>
     <x:row r="54">
       <x:c r="B54" s="26"/>
       <x:c r="C54" s="31"/>
       <x:c r="D54" s="31"/>
       <x:c r="E54" s="26"/>
-      <x:c r="G54" s="26"/>
-      <x:c r="H54" s="36"/>
+      <x:c r="H54" s="26"/>
+      <x:c r="I54" s="36"/>
     </x:row>
     <x:row r="55">
       <x:c r="B55" s="26"/>
       <x:c r="C55" s="31"/>
       <x:c r="D55" s="31"/>
       <x:c r="E55" s="26"/>
-      <x:c r="G55" s="26"/>
-      <x:c r="H55" s="36"/>
+      <x:c r="H55" s="26"/>
+      <x:c r="I55" s="36"/>
     </x:row>
     <x:row r="56">
       <x:c r="B56" s="26"/>
       <x:c r="C56" s="31"/>
       <x:c r="D56" s="31"/>
       <x:c r="E56" s="26"/>
-      <x:c r="G56" s="26"/>
-      <x:c r="H56" s="36"/>
+      <x:c r="H56" s="26"/>
+      <x:c r="I56" s="36"/>
     </x:row>
     <x:row r="57">
       <x:c r="B57" s="26"/>
       <x:c r="C57" s="31"/>
       <x:c r="D57" s="31"/>
       <x:c r="E57" s="26"/>
-      <x:c r="G57" s="26"/>
-      <x:c r="H57" s="36"/>
+      <x:c r="H57" s="26"/>
+      <x:c r="I57" s="36"/>
     </x:row>
     <x:row r="58">
       <x:c r="B58" s="26"/>
       <x:c r="C58" s="31"/>
       <x:c r="D58" s="31"/>
       <x:c r="E58" s="26"/>
-      <x:c r="G58" s="26"/>
-      <x:c r="H58" s="36"/>
+      <x:c r="H58" s="26"/>
+      <x:c r="I58" s="36"/>
     </x:row>
     <x:row r="59">
       <x:c r="B59" s="26"/>
       <x:c r="C59" s="31"/>
       <x:c r="D59" s="31"/>
       <x:c r="E59" s="26"/>
-      <x:c r="G59" s="26"/>
-      <x:c r="H59" s="36"/>
+      <x:c r="H59" s="26"/>
+      <x:c r="I59" s="36"/>
     </x:row>
     <x:row r="60">
       <x:c r="B60" s="26"/>
       <x:c r="C60" s="31"/>
       <x:c r="D60" s="31"/>
       <x:c r="E60" s="26"/>
-      <x:c r="G60" s="26"/>
-      <x:c r="H60" s="36"/>
+      <x:c r="H60" s="26"/>
+      <x:c r="I60" s="36"/>
     </x:row>
     <x:row r="61">
       <x:c r="B61" s="26"/>
       <x:c r="C61" s="31"/>
       <x:c r="D61" s="31"/>
       <x:c r="E61" s="26"/>
-      <x:c r="G61" s="26"/>
-      <x:c r="H61" s="36"/>
+      <x:c r="H61" s="26"/>
+      <x:c r="I61" s="36"/>
     </x:row>
     <x:row r="62">
       <x:c r="B62" s="26"/>
       <x:c r="C62" s="31"/>
       <x:c r="D62" s="31"/>
       <x:c r="E62" s="26"/>
-      <x:c r="G62" s="26"/>
-      <x:c r="H62" s="36"/>
+      <x:c r="H62" s="26"/>
+      <x:c r="I62" s="36"/>
     </x:row>
     <x:row r="63">
       <x:c r="B63" s="26"/>
       <x:c r="C63" s="31"/>
       <x:c r="D63" s="31"/>
       <x:c r="E63" s="26"/>
-      <x:c r="G63" s="26"/>
-      <x:c r="H63" s="36"/>
+      <x:c r="H63" s="26"/>
+      <x:c r="I63" s="36"/>
     </x:row>
     <x:row r="64">
       <x:c r="B64" s="26"/>
       <x:c r="C64" s="31"/>
       <x:c r="D64" s="31"/>
       <x:c r="E64" s="26"/>
-      <x:c r="G64" s="26"/>
-      <x:c r="H64" s="36"/>
+      <x:c r="H64" s="26"/>
+      <x:c r="I64" s="36"/>
     </x:row>
     <x:row r="65">
       <x:c r="B65" s="26"/>
       <x:c r="C65" s="31"/>
       <x:c r="D65" s="31"/>
       <x:c r="E65" s="26"/>
-      <x:c r="G65" s="26"/>
-      <x:c r="H65" s="36"/>
+      <x:c r="H65" s="26"/>
+      <x:c r="I65" s="36"/>
     </x:row>
     <x:row r="66">
       <x:c r="B66" s="26"/>
       <x:c r="C66" s="31"/>
       <x:c r="D66" s="31"/>
       <x:c r="E66" s="26"/>
-      <x:c r="G66" s="26"/>
-      <x:c r="H66" s="36"/>
+      <x:c r="H66" s="26"/>
+      <x:c r="I66" s="36"/>
     </x:row>
     <x:row r="67">
       <x:c r="B67" s="26"/>
       <x:c r="C67" s="31"/>
       <x:c r="D67" s="31"/>
       <x:c r="E67" s="26"/>
-      <x:c r="G67" s="26"/>
-      <x:c r="H67" s="36"/>
+      <x:c r="H67" s="26"/>
+      <x:c r="I67" s="36"/>
     </x:row>
     <x:row r="68">
       <x:c r="B68" s="26"/>
       <x:c r="C68" s="31"/>
       <x:c r="D68" s="31"/>
       <x:c r="E68" s="26"/>
-      <x:c r="G68" s="26"/>
-      <x:c r="H68" s="36"/>
+      <x:c r="H68" s="26"/>
+      <x:c r="I68" s="36"/>
     </x:row>
     <x:row r="69">
       <x:c r="B69" s="26"/>
       <x:c r="C69" s="31"/>
       <x:c r="D69" s="31"/>
       <x:c r="E69" s="26"/>
-      <x:c r="G69" s="26"/>
-      <x:c r="H69" s="36"/>
+      <x:c r="H69" s="26"/>
+      <x:c r="I69" s="36"/>
     </x:row>
     <x:row r="70">
       <x:c r="B70" s="26"/>
       <x:c r="C70" s="31"/>
       <x:c r="D70" s="31"/>
       <x:c r="E70" s="26"/>
-      <x:c r="G70" s="26"/>
-      <x:c r="H70" s="36"/>
+      <x:c r="H70" s="26"/>
+      <x:c r="I70" s="36"/>
     </x:row>
     <x:row r="71">
       <x:c r="B71" s="26"/>
       <x:c r="C71" s="31"/>
       <x:c r="D71" s="31"/>
       <x:c r="E71" s="26"/>
-      <x:c r="G71" s="26"/>
-      <x:c r="H71" s="36"/>
+      <x:c r="H71" s="26"/>
+      <x:c r="I71" s="36"/>
     </x:row>
     <x:row r="72">
       <x:c r="B72" s="26"/>
       <x:c r="C72" s="31"/>
       <x:c r="D72" s="31"/>
       <x:c r="E72" s="26"/>
-      <x:c r="G72" s="26"/>
-      <x:c r="H72" s="36"/>
+      <x:c r="H72" s="26"/>
+      <x:c r="I72" s="36"/>
     </x:row>
     <x:row r="73">
       <x:c r="B73" s="26"/>
       <x:c r="C73" s="31"/>
       <x:c r="D73" s="31"/>
       <x:c r="E73" s="26"/>
-      <x:c r="G73" s="26"/>
-      <x:c r="H73" s="36"/>
+      <x:c r="H73" s="26"/>
+      <x:c r="I73" s="36"/>
     </x:row>
     <x:row r="74">
       <x:c r="B74" s="26"/>
       <x:c r="C74" s="31"/>
       <x:c r="D74" s="31"/>
       <x:c r="E74" s="26"/>
-      <x:c r="G74" s="26"/>
-      <x:c r="H74" s="36"/>
+      <x:c r="H74" s="26"/>
+      <x:c r="I74" s="36"/>
     </x:row>
     <x:row r="75">
       <x:c r="B75" s="26"/>
       <x:c r="C75" s="31"/>
       <x:c r="D75" s="31"/>
       <x:c r="E75" s="26"/>
-      <x:c r="G75" s="26"/>
-      <x:c r="H75" s="36"/>
+      <x:c r="H75" s="26"/>
+      <x:c r="I75" s="36"/>
     </x:row>
     <x:row r="76">
       <x:c r="B76" s="26"/>
       <x:c r="C76" s="31"/>
       <x:c r="D76" s="31"/>
       <x:c r="E76" s="26"/>
-      <x:c r="G76" s="26"/>
-      <x:c r="H76" s="36"/>
+      <x:c r="H76" s="26"/>
+      <x:c r="I76" s="36"/>
     </x:row>
     <x:row r="77">
       <x:c r="B77" s="26"/>
       <x:c r="C77" s="31"/>
       <x:c r="D77" s="31"/>
       <x:c r="E77" s="26"/>
-      <x:c r="G77" s="26"/>
-      <x:c r="H77" s="36"/>
+      <x:c r="H77" s="26"/>
+      <x:c r="I77" s="36"/>
     </x:row>
     <x:row r="78">
       <x:c r="B78" s="26"/>
       <x:c r="C78" s="31"/>
       <x:c r="D78" s="31"/>
       <x:c r="E78" s="26"/>
-      <x:c r="G78" s="26"/>
-      <x:c r="H78" s="36"/>
+      <x:c r="H78" s="26"/>
+      <x:c r="I78" s="36"/>
     </x:row>
     <x:row r="79">
       <x:c r="B79" s="26"/>
       <x:c r="C79" s="31"/>
       <x:c r="D79" s="31"/>
       <x:c r="E79" s="26"/>
-      <x:c r="G79" s="26"/>
-      <x:c r="H79" s="36"/>
+      <x:c r="H79" s="26"/>
+      <x:c r="I79" s="36"/>
     </x:row>
     <x:row r="80">
       <x:c r="B80" s="26"/>
       <x:c r="C80" s="31"/>
       <x:c r="D80" s="31"/>
       <x:c r="E80" s="26"/>
-      <x:c r="G80" s="26"/>
-      <x:c r="H80" s="36"/>
+      <x:c r="H80" s="26"/>
+      <x:c r="I80" s="36"/>
     </x:row>
     <x:row r="81">
       <x:c r="B81" s="26"/>
       <x:c r="C81" s="31"/>
       <x:c r="D81" s="31"/>
       <x:c r="E81" s="26"/>
-      <x:c r="G81" s="26"/>
-      <x:c r="H81" s="36"/>
+      <x:c r="H81" s="26"/>
+      <x:c r="I81" s="36"/>
     </x:row>
     <x:row r="82">
       <x:c r="B82" s="26"/>
       <x:c r="C82" s="31"/>
       <x:c r="D82" s="31"/>
       <x:c r="E82" s="26"/>
-      <x:c r="G82" s="26"/>
-      <x:c r="H82" s="36"/>
+      <x:c r="H82" s="26"/>
+      <x:c r="I82" s="36"/>
     </x:row>
     <x:row r="83">
       <x:c r="B83" s="26"/>
       <x:c r="C83" s="31"/>
       <x:c r="D83" s="31"/>
       <x:c r="E83" s="26"/>
-      <x:c r="G83" s="26"/>
-      <x:c r="H83" s="36"/>
+      <x:c r="H83" s="26"/>
+      <x:c r="I83" s="36"/>
     </x:row>
     <x:row r="84">
       <x:c r="B84" s="26"/>
       <x:c r="C84" s="31"/>
       <x:c r="D84" s="31"/>
       <x:c r="E84" s="26"/>
-      <x:c r="G84" s="26"/>
-      <x:c r="H84" s="36"/>
+      <x:c r="H84" s="26"/>
+      <x:c r="I84" s="36"/>
     </x:row>
     <x:row r="85">
       <x:c r="B85" s="26"/>
       <x:c r="C85" s="31"/>
       <x:c r="D85" s="31"/>
       <x:c r="E85" s="26"/>
-      <x:c r="G85" s="26"/>
-      <x:c r="H85" s="36"/>
+      <x:c r="H85" s="26"/>
+      <x:c r="I85" s="36"/>
     </x:row>
     <x:row r="86">
       <x:c r="B86" s="26"/>
       <x:c r="C86" s="31"/>
       <x:c r="D86" s="31"/>
       <x:c r="E86" s="26"/>
-      <x:c r="G86" s="26"/>
-      <x:c r="H86" s="36"/>
+      <x:c r="H86" s="26"/>
+      <x:c r="I86" s="36"/>
     </x:row>
     <x:row r="87">
       <x:c r="B87" s="26"/>
       <x:c r="C87" s="31"/>
       <x:c r="D87" s="31"/>
       <x:c r="E87" s="26"/>
-      <x:c r="G87" s="26"/>
-      <x:c r="H87" s="36"/>
+      <x:c r="H87" s="26"/>
+      <x:c r="I87" s="36"/>
     </x:row>
     <x:row r="88">
       <x:c r="B88" s="26"/>
       <x:c r="C88" s="31"/>
       <x:c r="D88" s="31"/>
       <x:c r="E88" s="26"/>
-      <x:c r="G88" s="26"/>
-      <x:c r="H88" s="36"/>
+      <x:c r="H88" s="26"/>
+      <x:c r="I88" s="36"/>
     </x:row>
     <x:row r="89">
       <x:c r="B89" s="26"/>
       <x:c r="C89" s="31"/>
       <x:c r="D89" s="31"/>
       <x:c r="E89" s="26"/>
-      <x:c r="G89" s="26"/>
-      <x:c r="H89" s="36"/>
+      <x:c r="H89" s="26"/>
+      <x:c r="I89" s="36"/>
     </x:row>
     <x:row r="90">
       <x:c r="B90" s="26"/>
       <x:c r="C90" s="31"/>
       <x:c r="D90" s="31"/>
       <x:c r="E90" s="26"/>
-      <x:c r="G90" s="26"/>
-      <x:c r="H90" s="36"/>
+      <x:c r="H90" s="26"/>
+      <x:c r="I90" s="36"/>
     </x:row>
     <x:row r="91">
       <x:c r="B91" s="26"/>
       <x:c r="C91" s="31"/>
       <x:c r="D91" s="31"/>
       <x:c r="E91" s="26"/>
-      <x:c r="G91" s="26"/>
-      <x:c r="H91" s="36"/>
+      <x:c r="H91" s="26"/>
+      <x:c r="I91" s="36"/>
     </x:row>
     <x:row r="92">
       <x:c r="B92" s="26"/>
       <x:c r="C92" s="31"/>
       <x:c r="D92" s="31"/>
       <x:c r="E92" s="26"/>
-      <x:c r="G92" s="26"/>
-      <x:c r="H92" s="36"/>
+      <x:c r="H92" s="26"/>
+      <x:c r="I92" s="36"/>
     </x:row>
     <x:row r="93">
       <x:c r="B93" s="26"/>
       <x:c r="C93" s="31"/>
       <x:c r="D93" s="31"/>
       <x:c r="E93" s="26"/>
-      <x:c r="G93" s="26"/>
-      <x:c r="H93" s="36"/>
+      <x:c r="H93" s="26"/>
+      <x:c r="I93" s="36"/>
     </x:row>
     <x:row r="94">
       <x:c r="B94" s="26"/>
       <x:c r="C94" s="31"/>
       <x:c r="D94" s="31"/>
       <x:c r="E94" s="26"/>
-      <x:c r="G94" s="26"/>
-      <x:c r="H94" s="36"/>
+      <x:c r="H94" s="26"/>
+      <x:c r="I94" s="36"/>
     </x:row>
     <x:row r="95">
       <x:c r="B95" s="26"/>
       <x:c r="C95" s="31"/>
       <x:c r="D95" s="31"/>
       <x:c r="E95" s="26"/>
-      <x:c r="G95" s="26"/>
-      <x:c r="H95" s="36"/>
+      <x:c r="H95" s="26"/>
+      <x:c r="I95" s="36"/>
     </x:row>
     <x:row r="96">
       <x:c r="B96" s="26"/>
       <x:c r="C96" s="31"/>
       <x:c r="D96" s="31"/>
       <x:c r="E96" s="26"/>
-      <x:c r="G96" s="26"/>
-      <x:c r="H96" s="36"/>
+      <x:c r="H96" s="26"/>
+      <x:c r="I96" s="36"/>
     </x:row>
     <x:row r="97">
       <x:c r="B97" s="26"/>
       <x:c r="C97" s="31"/>
       <x:c r="D97" s="31"/>
       <x:c r="E97" s="26"/>
-      <x:c r="G97" s="26"/>
-      <x:c r="H97" s="36"/>
+      <x:c r="H97" s="26"/>
+      <x:c r="I97" s="36"/>
     </x:row>
     <x:row r="98">
       <x:c r="B98" s="26"/>
       <x:c r="C98" s="31"/>
       <x:c r="D98" s="31"/>
       <x:c r="E98" s="26"/>
-      <x:c r="G98" s="26"/>
-      <x:c r="H98" s="36"/>
+      <x:c r="H98" s="26"/>
+      <x:c r="I98" s="36"/>
     </x:row>
     <x:row r="99">
       <x:c r="B99" s="26"/>
       <x:c r="C99" s="31"/>
       <x:c r="D99" s="31"/>
       <x:c r="E99" s="26"/>
-      <x:c r="G99" s="26"/>
-      <x:c r="H99" s="36"/>
+      <x:c r="H99" s="26"/>
+      <x:c r="I99" s="36"/>
     </x:row>
     <x:row r="100">
       <x:c r="B100" s="26"/>
       <x:c r="C100" s="31"/>
       <x:c r="D100" s="31"/>
       <x:c r="E100" s="26"/>
-      <x:c r="G100" s="26"/>
-      <x:c r="H100" s="36"/>
+      <x:c r="H100" s="26"/>
+      <x:c r="I100" s="36"/>
     </x:row>
     <x:row r="101">
       <x:c r="B101" s="26"/>
       <x:c r="C101" s="31"/>
       <x:c r="D101" s="31"/>
       <x:c r="E101" s="26"/>
-      <x:c r="G101" s="26"/>
-      <x:c r="H101" s="36"/>
+      <x:c r="H101" s="26"/>
+      <x:c r="I101" s="36"/>
     </x:row>
     <x:row r="102">
       <x:c r="B102" s="26"/>
       <x:c r="C102" s="31"/>
       <x:c r="D102" s="31"/>
       <x:c r="E102" s="26"/>
-      <x:c r="G102" s="26"/>
-      <x:c r="H102" s="36"/>
+      <x:c r="H102" s="26"/>
+      <x:c r="I102" s="36"/>
     </x:row>
     <x:row r="103">
       <x:c r="B103" s="26"/>
       <x:c r="C103" s="31"/>
       <x:c r="D103" s="31"/>
       <x:c r="E103" s="26"/>
-      <x:c r="G103" s="26"/>
-      <x:c r="H103" s="36"/>
+      <x:c r="H103" s="26"/>
+      <x:c r="I103" s="36"/>
     </x:row>
     <x:row r="104">
       <x:c r="B104" s="26"/>
       <x:c r="C104" s="31"/>
       <x:c r="D104" s="31"/>
       <x:c r="E104" s="26"/>
-      <x:c r="G104" s="26"/>
-      <x:c r="H104" s="36"/>
+      <x:c r="H104" s="26"/>
+      <x:c r="I104" s="36"/>
     </x:row>
     <x:row r="105">
       <x:c r="B105" s="26"/>
       <x:c r="C105" s="31"/>
       <x:c r="D105" s="31"/>
       <x:c r="E105" s="26"/>
-      <x:c r="G105" s="26"/>
-      <x:c r="H105" s="36"/>
+      <x:c r="H105" s="26"/>
+      <x:c r="I105" s="36"/>
     </x:row>
     <x:row r="106">
       <x:c r="B106" s="26"/>
       <x:c r="C106" s="31"/>
       <x:c r="D106" s="31"/>
       <x:c r="E106" s="26"/>
-      <x:c r="G106" s="26"/>
-      <x:c r="H106" s="36"/>
+      <x:c r="H106" s="26"/>
+      <x:c r="I106" s="36"/>
     </x:row>
     <x:row r="107">
       <x:c r="B107" s="26"/>
       <x:c r="C107" s="31"/>
       <x:c r="D107" s="31"/>
       <x:c r="E107" s="26"/>
-      <x:c r="G107" s="26"/>
-      <x:c r="H107" s="36"/>
+      <x:c r="H107" s="26"/>
+      <x:c r="I107" s="36"/>
     </x:row>
     <x:row r="108">
       <x:c r="B108" s="26"/>
       <x:c r="C108" s="31"/>
       <x:c r="D108" s="31"/>
       <x:c r="E108" s="26"/>
-      <x:c r="G108" s="26"/>
-      <x:c r="H108" s="36"/>
+      <x:c r="H108" s="26"/>
+      <x:c r="I108" s="36"/>
     </x:row>
     <x:row r="109">
       <x:c r="B109" s="26"/>
       <x:c r="C109" s="31"/>
       <x:c r="D109" s="31"/>
       <x:c r="E109" s="26"/>
-      <x:c r="G109" s="26"/>
-      <x:c r="H109" s="36"/>
+      <x:c r="H109" s="26"/>
+      <x:c r="I109" s="36"/>
     </x:row>
     <x:row r="110">
       <x:c r="B110" s="26"/>
       <x:c r="C110" s="31"/>
       <x:c r="D110" s="31"/>
       <x:c r="E110" s="26"/>
-      <x:c r="G110" s="26"/>
-      <x:c r="H110" s="36"/>
+      <x:c r="H110" s="26"/>
+      <x:c r="I110" s="36"/>
     </x:row>
     <x:row r="111">
       <x:c r="B111" s="26"/>
       <x:c r="C111" s="31"/>
       <x:c r="D111" s="31"/>
       <x:c r="E111" s="26"/>
-      <x:c r="G111" s="26"/>
-      <x:c r="H111" s="36"/>
+      <x:c r="H111" s="26"/>
+      <x:c r="I111" s="36"/>
     </x:row>
     <x:row r="112">
       <x:c r="B112" s="26"/>
       <x:c r="C112" s="31"/>
       <x:c r="D112" s="31"/>
       <x:c r="E112" s="26"/>
-      <x:c r="G112" s="26"/>
-      <x:c r="H112" s="36"/>
+      <x:c r="H112" s="26"/>
+      <x:c r="I112" s="36"/>
     </x:row>
     <x:row r="113">
       <x:c r="B113" s="26"/>
       <x:c r="C113" s="31"/>
       <x:c r="D113" s="31"/>
       <x:c r="E113" s="26"/>
-      <x:c r="G113" s="26"/>
-      <x:c r="H113" s="36"/>
+      <x:c r="H113" s="26"/>
+      <x:c r="I113" s="36"/>
     </x:row>
     <x:row r="114">
       <x:c r="B114" s="26"/>
       <x:c r="C114" s="31"/>
       <x:c r="D114" s="31"/>
       <x:c r="E114" s="26"/>
-      <x:c r="G114" s="26"/>
-      <x:c r="H114" s="36"/>
+      <x:c r="H114" s="26"/>
+      <x:c r="I114" s="36"/>
     </x:row>
     <x:row r="115">
       <x:c r="B115" s="26"/>
       <x:c r="C115" s="31"/>
       <x:c r="D115" s="31"/>
       <x:c r="E115" s="26"/>
-      <x:c r="G115" s="26"/>
-      <x:c r="H115" s="36"/>
+      <x:c r="H115" s="26"/>
+      <x:c r="I115" s="36"/>
     </x:row>
     <x:row r="116">
       <x:c r="B116" s="26"/>
       <x:c r="C116" s="31"/>
       <x:c r="D116" s="31"/>
       <x:c r="E116" s="26"/>
-      <x:c r="G116" s="26"/>
-      <x:c r="H116" s="36"/>
+      <x:c r="H116" s="26"/>
+      <x:c r="I116" s="36"/>
     </x:row>
     <x:row r="117">
       <x:c r="B117" s="26"/>
       <x:c r="C117" s="31"/>
       <x:c r="D117" s="31"/>
       <x:c r="E117" s="26"/>
-      <x:c r="G117" s="26"/>
-      <x:c r="H117" s="36"/>
+      <x:c r="H117" s="26"/>
+      <x:c r="I117" s="36"/>
     </x:row>
     <x:row r="118">
       <x:c r="B118" s="26"/>
       <x:c r="C118" s="31"/>
       <x:c r="D118" s="31"/>
       <x:c r="E118" s="26"/>
-      <x:c r="G118" s="26"/>
-      <x:c r="H118" s="36"/>
+      <x:c r="H118" s="26"/>
+      <x:c r="I118" s="36"/>
     </x:row>
     <x:row r="119">
       <x:c r="B119" s="26"/>
       <x:c r="C119" s="31"/>
       <x:c r="D119" s="31"/>
       <x:c r="E119" s="26"/>
-      <x:c r="G119" s="26"/>
-      <x:c r="H119" s="36"/>
+      <x:c r="H119" s="26"/>
+      <x:c r="I119" s="36"/>
     </x:row>
     <x:row r="120">
       <x:c r="B120" s="26"/>
       <x:c r="C120" s="31"/>
       <x:c r="D120" s="31"/>
       <x:c r="E120" s="26"/>
-      <x:c r="G120" s="26"/>
-      <x:c r="H120" s="36"/>
+      <x:c r="H120" s="26"/>
+      <x:c r="I120" s="36"/>
     </x:row>
     <x:row r="121">
       <x:c r="B121" s="26"/>
       <x:c r="C121" s="31"/>
       <x:c r="D121" s="31"/>
       <x:c r="E121" s="26"/>
-      <x:c r="G121" s="26"/>
-      <x:c r="H121" s="36"/>
+      <x:c r="H121" s="26"/>
+      <x:c r="I121" s="36"/>
     </x:row>
     <x:row r="122">
       <x:c r="B122" s="26"/>
       <x:c r="C122" s="31"/>
       <x:c r="D122" s="31"/>
       <x:c r="E122" s="26"/>
-      <x:c r="G122" s="26"/>
-      <x:c r="H122" s="36"/>
+      <x:c r="H122" s="26"/>
+      <x:c r="I122" s="36"/>
     </x:row>
     <x:row r="123">
       <x:c r="B123" s="26"/>
       <x:c r="C123" s="31"/>
       <x:c r="D123" s="31"/>
       <x:c r="E123" s="26"/>
-      <x:c r="G123" s="26"/>
-      <x:c r="H123" s="36"/>
+      <x:c r="H123" s="26"/>
+      <x:c r="I123" s="36"/>
     </x:row>
     <x:row r="124">
       <x:c r="B124" s="26"/>
       <x:c r="C124" s="31"/>
       <x:c r="D124" s="31"/>
       <x:c r="E124" s="26"/>
-      <x:c r="G124" s="26"/>
-      <x:c r="H124" s="36"/>
+      <x:c r="H124" s="26"/>
+      <x:c r="I124" s="36"/>
     </x:row>
     <x:row r="125">
       <x:c r="B125" s="26"/>
       <x:c r="C125" s="31"/>
       <x:c r="D125" s="31"/>
       <x:c r="E125" s="26"/>
-      <x:c r="G125" s="26"/>
-      <x:c r="H125" s="36"/>
+      <x:c r="H125" s="26"/>
+      <x:c r="I125" s="36"/>
     </x:row>
     <x:row r="126">
       <x:c r="B126" s="26"/>
       <x:c r="C126" s="31"/>
       <x:c r="D126" s="31"/>
       <x:c r="E126" s="26"/>
-      <x:c r="G126" s="26"/>
-      <x:c r="H126" s="36"/>
+      <x:c r="H126" s="26"/>
+      <x:c r="I126" s="36"/>
     </x:row>
     <x:row r="127">
       <x:c r="B127" s="26"/>
       <x:c r="C127" s="31"/>
       <x:c r="D127" s="31"/>
       <x:c r="E127" s="26"/>
-      <x:c r="G127" s="26"/>
-      <x:c r="H127" s="36"/>
+      <x:c r="H127" s="26"/>
+      <x:c r="I127" s="36"/>
     </x:row>
     <x:row r="128">
       <x:c r="B128" s="26"/>
       <x:c r="C128" s="31"/>
       <x:c r="D128" s="31"/>
       <x:c r="E128" s="26"/>
-      <x:c r="G128" s="26"/>
-      <x:c r="H128" s="36"/>
+      <x:c r="H128" s="26"/>
+      <x:c r="I128" s="36"/>
     </x:row>
     <x:row r="129">
       <x:c r="B129" s="26"/>
       <x:c r="C129" s="31"/>
       <x:c r="D129" s="31"/>
       <x:c r="E129" s="26"/>
-      <x:c r="G129" s="26"/>
-      <x:c r="H129" s="36"/>
+      <x:c r="H129" s="26"/>
+      <x:c r="I129" s="36"/>
     </x:row>
     <x:row r="130">
       <x:c r="B130" s="26"/>
       <x:c r="C130" s="31"/>
       <x:c r="D130" s="31"/>
       <x:c r="E130" s="26"/>
-      <x:c r="G130" s="26"/>
-      <x:c r="H130" s="36"/>
+      <x:c r="H130" s="26"/>
+      <x:c r="I130" s="36"/>
     </x:row>
     <x:row r="131">
       <x:c r="B131" s="26"/>
       <x:c r="C131" s="31"/>
       <x:c r="D131" s="31"/>
       <x:c r="E131" s="26"/>
-      <x:c r="G131" s="26"/>
-      <x:c r="H131" s="36"/>
+      <x:c r="H131" s="26"/>
+      <x:c r="I131" s="36"/>
     </x:row>
     <x:row r="132">
       <x:c r="B132" s="26"/>
       <x:c r="C132" s="31"/>
       <x:c r="D132" s="31"/>
       <x:c r="E132" s="26"/>
-      <x:c r="G132" s="26"/>
-      <x:c r="H132" s="36"/>
+      <x:c r="H132" s="26"/>
+      <x:c r="I132" s="36"/>
     </x:row>
     <x:row r="133">
       <x:c r="B133" s="26"/>
       <x:c r="C133" s="31"/>
       <x:c r="D133" s="31"/>
       <x:c r="E133" s="26"/>
-      <x:c r="G133" s="26"/>
-      <x:c r="H133" s="36"/>
+      <x:c r="H133" s="26"/>
+      <x:c r="I133" s="36"/>
     </x:row>
     <x:row r="134">
       <x:c r="B134" s="26"/>
       <x:c r="C134" s="31"/>
       <x:c r="D134" s="31"/>
       <x:c r="E134" s="26"/>
-      <x:c r="G134" s="26"/>
-      <x:c r="H134" s="36"/>
+      <x:c r="H134" s="26"/>
+      <x:c r="I134" s="36"/>
     </x:row>
     <x:row r="135">
       <x:c r="B135" s="26"/>
       <x:c r="C135" s="31"/>
       <x:c r="D135" s="31"/>
       <x:c r="E135" s="26"/>
-      <x:c r="G135" s="26"/>
-      <x:c r="H135" s="36"/>
+      <x:c r="H135" s="26"/>
+      <x:c r="I135" s="36"/>
     </x:row>
     <x:row r="136">
       <x:c r="B136" s="26"/>
       <x:c r="C136" s="31"/>
       <x:c r="D136" s="31"/>
       <x:c r="E136" s="26"/>
-      <x:c r="G136" s="26"/>
-      <x:c r="H136" s="36"/>
+      <x:c r="H136" s="26"/>
+      <x:c r="I136" s="36"/>
     </x:row>
     <x:row r="137">
       <x:c r="B137" s="26"/>
       <x:c r="C137" s="31"/>
       <x:c r="D137" s="31"/>
       <x:c r="E137" s="26"/>
-      <x:c r="G137" s="26"/>
-      <x:c r="H137" s="36"/>
+      <x:c r="H137" s="26"/>
+      <x:c r="I137" s="36"/>
     </x:row>
     <x:row r="138">
       <x:c r="B138" s="26"/>
       <x:c r="C138" s="31"/>
       <x:c r="D138" s="31"/>
       <x:c r="E138" s="26"/>
-      <x:c r="G138" s="26"/>
-      <x:c r="H138" s="36"/>
+      <x:c r="H138" s="26"/>
+      <x:c r="I138" s="36"/>
     </x:row>
     <x:row r="139">
       <x:c r="B139" s="26"/>
       <x:c r="C139" s="31"/>
       <x:c r="D139" s="31"/>
       <x:c r="E139" s="26"/>
-      <x:c r="G139" s="26"/>
-      <x:c r="H139" s="36"/>
+      <x:c r="H139" s="26"/>
+      <x:c r="I139" s="36"/>
     </x:row>
     <x:row r="140">
       <x:c r="B140" s="26"/>
       <x:c r="C140" s="31"/>
       <x:c r="D140" s="31"/>
       <x:c r="E140" s="26"/>
-      <x:c r="G140" s="26"/>
-      <x:c r="H140" s="36"/>
+      <x:c r="H140" s="26"/>
+      <x:c r="I140" s="36"/>
     </x:row>
     <x:row r="141">
       <x:c r="B141" s="26"/>
       <x:c r="C141" s="31"/>
       <x:c r="D141" s="31"/>
       <x:c r="E141" s="26"/>
-      <x:c r="G141" s="26"/>
-      <x:c r="H141" s="36"/>
+      <x:c r="H141" s="26"/>
+      <x:c r="I141" s="36"/>
     </x:row>
     <x:row r="142">
       <x:c r="B142" s="26"/>
       <x:c r="C142" s="31"/>
       <x:c r="D142" s="31"/>
       <x:c r="E142" s="26"/>
-      <x:c r="G142" s="26"/>
-      <x:c r="H142" s="36"/>
+      <x:c r="H142" s="26"/>
+      <x:c r="I142" s="36"/>
     </x:row>
     <x:row r="143">
       <x:c r="B143" s="26"/>
       <x:c r="C143" s="31"/>
       <x:c r="D143" s="31"/>
       <x:c r="E143" s="26"/>
-      <x:c r="G143" s="26"/>
-      <x:c r="H143" s="36"/>
+      <x:c r="H143" s="26"/>
+      <x:c r="I143" s="36"/>
     </x:row>
     <x:row r="144">
       <x:c r="B144" s="26"/>
       <x:c r="C144" s="31"/>
       <x:c r="D144" s="31"/>
       <x:c r="E144" s="26"/>
-      <x:c r="G144" s="26"/>
-      <x:c r="H144" s="36"/>
+      <x:c r="H144" s="26"/>
+      <x:c r="I144" s="36"/>
     </x:row>
     <x:row r="145">
       <x:c r="B145" s="26"/>
       <x:c r="C145" s="31"/>
       <x:c r="D145" s="31"/>
       <x:c r="E145" s="26"/>
-      <x:c r="G145" s="26"/>
-      <x:c r="H145" s="36"/>
+      <x:c r="H145" s="26"/>
+      <x:c r="I145" s="36"/>
     </x:row>
     <x:row r="146">
       <x:c r="B146" s="26"/>
       <x:c r="C146" s="31"/>
       <x:c r="D146" s="31"/>
       <x:c r="E146" s="26"/>
-      <x:c r="G146" s="26"/>
-      <x:c r="H146" s="36"/>
+      <x:c r="H146" s="26"/>
+      <x:c r="I146" s="36"/>
     </x:row>
     <x:row r="147">
       <x:c r="B147" s="26"/>
       <x:c r="C147" s="31"/>
       <x:c r="D147" s="31"/>
       <x:c r="E147" s="26"/>
-      <x:c r="G147" s="26"/>
-      <x:c r="H147" s="36"/>
+      <x:c r="H147" s="26"/>
+      <x:c r="I147" s="36"/>
     </x:row>
     <x:row r="148">
       <x:c r="B148" s="26"/>
       <x:c r="C148" s="31"/>
       <x:c r="D148" s="31"/>
       <x:c r="E148" s="26"/>
-      <x:c r="G148" s="26"/>
-      <x:c r="H148" s="36"/>
+      <x:c r="H148" s="26"/>
+      <x:c r="I148" s="36"/>
     </x:row>
     <x:row r="149">
       <x:c r="B149" s="26"/>
       <x:c r="C149" s="31"/>
       <x:c r="D149" s="31"/>
       <x:c r="E149" s="26"/>
-      <x:c r="G149" s="26"/>
-      <x:c r="H149" s="36"/>
+      <x:c r="H149" s="26"/>
+      <x:c r="I149" s="36"/>
     </x:row>
     <x:row r="150">
       <x:c r="B150" s="26"/>
       <x:c r="C150" s="31"/>
       <x:c r="D150" s="31"/>
       <x:c r="E150" s="26"/>
-      <x:c r="G150" s="26"/>
-      <x:c r="H150" s="36"/>
+      <x:c r="H150" s="26"/>
+      <x:c r="I150" s="36"/>
     </x:row>
     <x:row r="151">
       <x:c r="B151" s="26"/>
       <x:c r="C151" s="31"/>
       <x:c r="D151" s="31"/>
       <x:c r="E151" s="26"/>
-      <x:c r="G151" s="26"/>
-      <x:c r="H151" s="36"/>
+      <x:c r="H151" s="26"/>
+      <x:c r="I151" s="36"/>
     </x:row>
     <x:row r="152">
       <x:c r="B152" s="26"/>
       <x:c r="C152" s="31"/>
       <x:c r="D152" s="31"/>
       <x:c r="E152" s="26"/>
-      <x:c r="G152" s="26"/>
-      <x:c r="H152" s="36"/>
+      <x:c r="H152" s="26"/>
+      <x:c r="I152" s="36"/>
     </x:row>
     <x:row r="153">
       <x:c r="B153" s="26"/>
       <x:c r="C153" s="31"/>
       <x:c r="D153" s="31"/>
       <x:c r="E153" s="26"/>
-      <x:c r="G153" s="26"/>
-      <x:c r="H153" s="36"/>
+      <x:c r="H153" s="26"/>
+      <x:c r="I153" s="36"/>
     </x:row>
     <x:row r="154">
       <x:c r="B154" s="26"/>
       <x:c r="C154" s="31"/>
       <x:c r="D154" s="31"/>
       <x:c r="E154" s="26"/>
-      <x:c r="G154" s="26"/>
-      <x:c r="H154" s="36"/>
+      <x:c r="H154" s="26"/>
+      <x:c r="I154" s="36"/>
     </x:row>
     <x:row r="155">
       <x:c r="B155" s="26"/>
       <x:c r="C155" s="31"/>
       <x:c r="D155" s="31"/>
       <x:c r="E155" s="26"/>
-      <x:c r="G155" s="26"/>
-      <x:c r="H155" s="36"/>
+      <x:c r="H155" s="26"/>
+      <x:c r="I155" s="36"/>
     </x:row>
     <x:row r="156">
       <x:c r="B156" s="26"/>
       <x:c r="C156" s="31"/>
       <x:c r="D156" s="31"/>
       <x:c r="E156" s="26"/>
-      <x:c r="G156" s="26"/>
-      <x:c r="H156" s="36"/>
+      <x:c r="H156" s="26"/>
+      <x:c r="I156" s="36"/>
     </x:row>
     <x:row r="157">
       <x:c r="B157" s="26"/>
       <x:c r="C157" s="31"/>
       <x:c r="D157" s="31"/>
       <x:c r="E157" s="26"/>
-      <x:c r="G157" s="26"/>
-      <x:c r="H157" s="36"/>
+      <x:c r="H157" s="26"/>
+      <x:c r="I157" s="36"/>
     </x:row>
     <x:row r="158">
       <x:c r="B158" s="26"/>
       <x:c r="C158" s="31"/>
       <x:c r="D158" s="31"/>
       <x:c r="E158" s="26"/>
-      <x:c r="G158" s="26"/>
-      <x:c r="H158" s="36"/>
+      <x:c r="H158" s="26"/>
+      <x:c r="I158" s="36"/>
     </x:row>
     <x:row r="159">
       <x:c r="B159" s="26"/>
       <x:c r="C159" s="31"/>
       <x:c r="D159" s="31"/>
       <x:c r="E159" s="26"/>
-      <x:c r="G159" s="26"/>
-      <x:c r="H159" s="36"/>
+      <x:c r="H159" s="26"/>
+      <x:c r="I159" s="36"/>
     </x:row>
     <x:row r="160">
       <x:c r="B160" s="26"/>
       <x:c r="C160" s="31"/>
       <x:c r="D160" s="31"/>
       <x:c r="E160" s="26"/>
-      <x:c r="G160" s="26"/>
-      <x:c r="H160" s="36"/>
+      <x:c r="H160" s="26"/>
+      <x:c r="I160" s="36"/>
     </x:row>
     <x:row r="161">
       <x:c r="B161" s="26"/>
       <x:c r="C161" s="31"/>
       <x:c r="D161" s="31"/>
       <x:c r="E161" s="26"/>
-      <x:c r="G161" s="26"/>
-      <x:c r="H161" s="36"/>
+      <x:c r="H161" s="26"/>
+      <x:c r="I161" s="36"/>
     </x:row>
     <x:row r="162">
       <x:c r="B162" s="26"/>
       <x:c r="C162" s="31"/>
       <x:c r="D162" s="31"/>
       <x:c r="E162" s="26"/>
-      <x:c r="G162" s="26"/>
-      <x:c r="H162" s="36"/>
+      <x:c r="H162" s="26"/>
+      <x:c r="I162" s="36"/>
     </x:row>
     <x:row r="163">
       <x:c r="B163" s="26"/>
       <x:c r="C163" s="31"/>
       <x:c r="D163" s="31"/>
       <x:c r="E163" s="26"/>
-      <x:c r="G163" s="26"/>
-      <x:c r="H163" s="36"/>
+      <x:c r="H163" s="26"/>
+      <x:c r="I163" s="36"/>
     </x:row>
     <x:row r="164">
       <x:c r="B164" s="26"/>
       <x:c r="C164" s="31"/>
       <x:c r="D164" s="31"/>
       <x:c r="E164" s="26"/>
-      <x:c r="G164" s="26"/>
-      <x:c r="H164" s="36"/>
+      <x:c r="H164" s="26"/>
+      <x:c r="I164" s="36"/>
     </x:row>
     <x:row r="165">
       <x:c r="B165" s="26"/>
       <x:c r="C165" s="31"/>
       <x:c r="D165" s="31"/>
       <x:c r="E165" s="26"/>
-      <x:c r="G165" s="26"/>
-      <x:c r="H165" s="36"/>
+      <x:c r="H165" s="26"/>
+      <x:c r="I165" s="36"/>
     </x:row>
     <x:row r="166">
       <x:c r="B166" s="26"/>
       <x:c r="C166" s="31"/>
       <x:c r="D166" s="31"/>
       <x:c r="E166" s="26"/>
-      <x:c r="G166" s="26"/>
-      <x:c r="H166" s="36"/>
+      <x:c r="H166" s="26"/>
+      <x:c r="I166" s="36"/>
     </x:row>
     <x:row r="167">
       <x:c r="B167" s="26"/>
       <x:c r="C167" s="31"/>
       <x:c r="D167" s="31"/>
       <x:c r="E167" s="26"/>
-      <x:c r="G167" s="26"/>
-      <x:c r="H167" s="36"/>
+      <x:c r="H167" s="26"/>
+      <x:c r="I167" s="36"/>
     </x:row>
     <x:row r="168">
       <x:c r="B168" s="26"/>
       <x:c r="C168" s="31"/>
       <x:c r="D168" s="31"/>
       <x:c r="E168" s="26"/>
-      <x:c r="G168" s="26"/>
-      <x:c r="H168" s="36"/>
+      <x:c r="H168" s="26"/>
+      <x:c r="I168" s="36"/>
     </x:row>
     <x:row r="169">
       <x:c r="B169" s="26"/>
       <x:c r="C169" s="31"/>
       <x:c r="D169" s="31"/>
       <x:c r="E169" s="26"/>
-      <x:c r="G169" s="26"/>
-      <x:c r="H169" s="36"/>
+      <x:c r="H169" s="26"/>
+      <x:c r="I169" s="36"/>
     </x:row>
     <x:row r="170">
       <x:c r="B170" s="26"/>
       <x:c r="C170" s="31"/>
       <x:c r="D170" s="31"/>
       <x:c r="E170" s="26"/>
-      <x:c r="G170" s="26"/>
-      <x:c r="H170" s="36"/>
+      <x:c r="H170" s="26"/>
+      <x:c r="I170" s="36"/>
     </x:row>
     <x:row r="171">
       <x:c r="B171" s="26"/>
       <x:c r="C171" s="31"/>
       <x:c r="D171" s="31"/>
       <x:c r="E171" s="26"/>
-      <x:c r="G171" s="26"/>
-      <x:c r="H171" s="36"/>
+      <x:c r="H171" s="26"/>
+      <x:c r="I171" s="36"/>
     </x:row>
     <x:row r="172">
       <x:c r="B172" s="26"/>
       <x:c r="C172" s="31"/>
       <x:c r="D172" s="31"/>
       <x:c r="E172" s="26"/>
-      <x:c r="G172" s="26"/>
-      <x:c r="H172" s="36"/>
+      <x:c r="H172" s="26"/>
+      <x:c r="I172" s="36"/>
     </x:row>
     <x:row r="173">
       <x:c r="B173" s="26"/>
       <x:c r="C173" s="31"/>
       <x:c r="D173" s="31"/>
       <x:c r="E173" s="26"/>
-      <x:c r="G173" s="26"/>
-      <x:c r="H173" s="36"/>
+      <x:c r="H173" s="26"/>
+      <x:c r="I173" s="36"/>
     </x:row>
     <x:row r="174">
       <x:c r="B174" s="26"/>
       <x:c r="C174" s="31"/>
       <x:c r="D174" s="31"/>
       <x:c r="E174" s="26"/>
-      <x:c r="G174" s="26"/>
-      <x:c r="H174" s="36"/>
+      <x:c r="H174" s="26"/>
+      <x:c r="I174" s="36"/>
     </x:row>
     <x:row r="175">
       <x:c r="B175" s="26"/>
       <x:c r="C175" s="31"/>
       <x:c r="D175" s="31"/>
       <x:c r="E175" s="26"/>
-      <x:c r="G175" s="26"/>
-      <x:c r="H175" s="36"/>
+      <x:c r="H175" s="26"/>
+      <x:c r="I175" s="36"/>
     </x:row>
     <x:row r="176">
       <x:c r="B176" s="26"/>
       <x:c r="C176" s="31"/>
       <x:c r="D176" s="31"/>
       <x:c r="E176" s="26"/>
-      <x:c r="G176" s="26"/>
-      <x:c r="H176" s="36"/>
+      <x:c r="H176" s="26"/>
+      <x:c r="I176" s="36"/>
     </x:row>
     <x:row r="177">
       <x:c r="B177" s="26"/>
       <x:c r="C177" s="31"/>
       <x:c r="D177" s="31"/>
       <x:c r="E177" s="26"/>
-      <x:c r="G177" s="26"/>
-      <x:c r="H177" s="36"/>
+      <x:c r="H177" s="26"/>
+      <x:c r="I177" s="36"/>
     </x:row>
     <x:row r="178">
       <x:c r="B178" s="26"/>
       <x:c r="C178" s="31"/>
       <x:c r="D178" s="31"/>
       <x:c r="E178" s="26"/>
-      <x:c r="G178" s="26"/>
-      <x:c r="H178" s="36"/>
+      <x:c r="H178" s="26"/>
+      <x:c r="I178" s="36"/>
     </x:row>
     <x:row r="179">
       <x:c r="B179" s="26"/>
       <x:c r="C179" s="31"/>
       <x:c r="D179" s="31"/>
       <x:c r="E179" s="26"/>
-      <x:c r="G179" s="26"/>
-      <x:c r="H179" s="36"/>
+      <x:c r="H179" s="26"/>
+      <x:c r="I179" s="36"/>
     </x:row>
     <x:row r="180">
       <x:c r="B180" s="26"/>
       <x:c r="C180" s="31"/>
       <x:c r="D180" s="31"/>
       <x:c r="E180" s="26"/>
-      <x:c r="G180" s="26"/>
-      <x:c r="H180" s="36"/>
+      <x:c r="H180" s="26"/>
+      <x:c r="I180" s="36"/>
     </x:row>
     <x:row r="181">
       <x:c r="B181" s="26"/>
       <x:c r="C181" s="31"/>
       <x:c r="D181" s="31"/>
       <x:c r="E181" s="26"/>
-      <x:c r="G181" s="26"/>
-      <x:c r="H181" s="36"/>
+      <x:c r="H181" s="26"/>
+      <x:c r="I181" s="36"/>
     </x:row>
     <x:row r="182">
       <x:c r="B182" s="26"/>
       <x:c r="C182" s="31"/>
       <x:c r="D182" s="31"/>
       <x:c r="E182" s="26"/>
-      <x:c r="G182" s="26"/>
-      <x:c r="H182" s="36"/>
+      <x:c r="H182" s="26"/>
+      <x:c r="I182" s="36"/>
     </x:row>
     <x:row r="183">
       <x:c r="B183" s="26"/>
       <x:c r="C183" s="31"/>
       <x:c r="D183" s="31"/>
       <x:c r="E183" s="26"/>
-      <x:c r="G183" s="26"/>
-      <x:c r="H183" s="36"/>
+      <x:c r="H183" s="26"/>
+      <x:c r="I183" s="36"/>
     </x:row>
     <x:row r="184">
       <x:c r="B184" s="26"/>
       <x:c r="C184" s="31"/>
       <x:c r="D184" s="31"/>
       <x:c r="E184" s="26"/>
-      <x:c r="G184" s="26"/>
-      <x:c r="H184" s="36"/>
+      <x:c r="H184" s="26"/>
+      <x:c r="I184" s="36"/>
     </x:row>
     <x:row r="185">
       <x:c r="B185" s="26"/>
       <x:c r="C185" s="31"/>
       <x:c r="D185" s="31"/>
       <x:c r="E185" s="26"/>
-      <x:c r="G185" s="26"/>
-      <x:c r="H185" s="36"/>
+      <x:c r="H185" s="26"/>
+      <x:c r="I185" s="36"/>
     </x:row>
     <x:row r="186">
       <x:c r="B186" s="26"/>
       <x:c r="C186" s="31"/>
       <x:c r="D186" s="31"/>
       <x:c r="E186" s="26"/>
-      <x:c r="G186" s="26"/>
-      <x:c r="H186" s="36"/>
+      <x:c r="H186" s="26"/>
+      <x:c r="I186" s="36"/>
     </x:row>
     <x:row r="187">
       <x:c r="B187" s="26"/>
       <x:c r="C187" s="31"/>
       <x:c r="D187" s="31"/>
       <x:c r="E187" s="26"/>
-      <x:c r="G187" s="26"/>
-      <x:c r="H187" s="36"/>
+      <x:c r="H187" s="26"/>
+      <x:c r="I187" s="36"/>
     </x:row>
     <x:row r="188">
       <x:c r="B188" s="26"/>
       <x:c r="C188" s="31"/>
       <x:c r="D188" s="31"/>
       <x:c r="E188" s="26"/>
-      <x:c r="G188" s="26"/>
-      <x:c r="H188" s="36"/>
+      <x:c r="H188" s="26"/>
+      <x:c r="I188" s="36"/>
     </x:row>
     <x:row r="189">
       <x:c r="B189" s="26"/>
       <x:c r="C189" s="31"/>
       <x:c r="D189" s="31"/>
       <x:c r="E189" s="26"/>
-      <x:c r="G189" s="26"/>
-      <x:c r="H189" s="36"/>
+      <x:c r="H189" s="26"/>
+      <x:c r="I189" s="36"/>
     </x:row>
     <x:row r="190">
       <x:c r="B190" s="26"/>
       <x:c r="C190" s="31"/>
       <x:c r="D190" s="31"/>
       <x:c r="E190" s="26"/>
-      <x:c r="G190" s="26"/>
-      <x:c r="H190" s="36"/>
+      <x:c r="H190" s="26"/>
+      <x:c r="I190" s="36"/>
     </x:row>
     <x:row r="191">
       <x:c r="B191" s="26"/>
       <x:c r="C191" s="31"/>
       <x:c r="D191" s="31"/>
       <x:c r="E191" s="26"/>
-      <x:c r="G191" s="26"/>
-      <x:c r="H191" s="36"/>
+      <x:c r="H191" s="26"/>
+      <x:c r="I191" s="36"/>
     </x:row>
     <x:row r="192">
       <x:c r="B192" s="26"/>
       <x:c r="C192" s="31"/>
       <x:c r="D192" s="31"/>
       <x:c r="E192" s="26"/>
-      <x:c r="G192" s="26"/>
-      <x:c r="H192" s="36"/>
+      <x:c r="H192" s="26"/>
+      <x:c r="I192" s="36"/>
     </x:row>
     <x:row r="193">
       <x:c r="B193" s="26"/>
       <x:c r="C193" s="31"/>
       <x:c r="D193" s="31"/>
       <x:c r="E193" s="26"/>
-      <x:c r="G193" s="26"/>
-      <x:c r="H193" s="36"/>
+      <x:c r="H193" s="26"/>
+      <x:c r="I193" s="36"/>
     </x:row>
     <x:row r="194">
       <x:c r="B194" s="26"/>
       <x:c r="C194" s="31"/>
       <x:c r="D194" s="31"/>
       <x:c r="E194" s="26"/>
-      <x:c r="G194" s="26"/>
-      <x:c r="H194" s="36"/>
+      <x:c r="H194" s="26"/>
+      <x:c r="I194" s="36"/>
     </x:row>
     <x:row r="195">
       <x:c r="B195" s="26"/>
       <x:c r="C195" s="31"/>
       <x:c r="D195" s="31"/>
       <x:c r="E195" s="26"/>
-      <x:c r="G195" s="26"/>
-      <x:c r="H195" s="36"/>
+      <x:c r="H195" s="26"/>
+      <x:c r="I195" s="36"/>
     </x:row>
     <x:row r="196">
       <x:c r="B196" s="26"/>
       <x:c r="C196" s="31"/>
       <x:c r="D196" s="31"/>
       <x:c r="E196" s="26"/>
-      <x:c r="G196" s="26"/>
-      <x:c r="H196" s="36"/>
+      <x:c r="H196" s="26"/>
+      <x:c r="I196" s="36"/>
     </x:row>
     <x:row r="197">
       <x:c r="B197" s="26"/>
       <x:c r="C197" s="31"/>
       <x:c r="D197" s="31"/>
       <x:c r="E197" s="26"/>
-      <x:c r="G197" s="26"/>
-      <x:c r="H197" s="36"/>
+      <x:c r="H197" s="26"/>
+      <x:c r="I197" s="36"/>
     </x:row>
     <x:row r="198">
       <x:c r="B198" s="26"/>
       <x:c r="C198" s="31"/>
       <x:c r="D198" s="31"/>
       <x:c r="E198" s="26"/>
-      <x:c r="G198" s="26"/>
-      <x:c r="H198" s="36"/>
+      <x:c r="H198" s="26"/>
+      <x:c r="I198" s="36"/>
     </x:row>
     <x:row r="199">
       <x:c r="B199" s="26"/>
       <x:c r="C199" s="31"/>
       <x:c r="D199" s="31"/>
       <x:c r="E199" s="26"/>
-      <x:c r="G199" s="26"/>
-      <x:c r="H199" s="36"/>
+      <x:c r="H199" s="26"/>
+      <x:c r="I199" s="36"/>
     </x:row>
     <x:row r="200">
       <x:c r="B200" s="26"/>
       <x:c r="C200" s="31"/>
       <x:c r="D200" s="31"/>
       <x:c r="E200" s="26"/>
-      <x:c r="G200" s="26"/>
-      <x:c r="H200" s="36"/>
+      <x:c r="H200" s="26"/>
+      <x:c r="I200" s="36"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F200">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="已到港已卸船"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="已到港未卸船"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I2:I200">
+  <x:conditionalFormatting sqref="J2:J200">
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="失败"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="已完成"/>
   </x:conditionalFormatting>
@@ -2447,13 +2467,13 @@
     <x:dataValidation type="list" sqref="F2:F200">
       <x:formula1>"未到港未卸船,已到港未卸船,已到港已卸船"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I200">
+    <x:dataValidation type="list" sqref="J2:J200">
       <x:formula1>"待查询,查询中,已完成,失败"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc150887f7ff4bfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redfb2895ef664c65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2798,7 +2818,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fcae2c6be8a4636"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdee02dd4e21d4d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>